<commit_message>
fixed some fronted bugs
</commit_message>
<xml_diff>
--- a/Intern Tracker.xlsx
+++ b/Intern Tracker.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21000" windowHeight="8745"/>
+    <workbookView windowWidth="24000" windowHeight="9615"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276">
   <si>
     <t>PROJECT</t>
   </si>
@@ -359,6 +359,27 @@
   </si>
   <si>
     <t>Added a "preview-only" mode that lets the system fetch raw text without needing to generate a full Word file</t>
+  </si>
+  <si>
+    <t>Preview Session Control</t>
+  </si>
+  <si>
+    <t>Fixed the preview pane that used to diasppear on refresh</t>
+  </si>
+  <si>
+    <t>separated the confirm and download feature by separating apis and creating separate download api</t>
+  </si>
+  <si>
+    <t>added version history</t>
+  </si>
+  <si>
+    <t>added version history feature for comapring between the document versions</t>
+  </si>
+  <si>
+    <t>fixed the avg time bug</t>
+  </si>
+  <si>
+    <t>separating apis led for blank avg time bug so fixed the blank avg time bug</t>
   </si>
   <si>
     <t>Date</t>
@@ -854,10 +875,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="176" formatCode="_ &quot;₹&quot;\ * #,##0_ ;_ &quot;₹&quot;\ * \-#,##0_ ;_ &quot;₹&quot;\ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ &quot;₹&quot;\ * #,##0_ ;_ &quot;₹&quot;\ * \-#,##0_ ;_ &quot;₹&quot;\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="180" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="28">
@@ -916,6 +937,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -923,21 +951,22 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -952,10 +981,26 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -967,16 +1012,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -999,16 +1036,30 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1021,39 +1072,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1110,19 +1131,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1134,19 +1143,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1158,55 +1179,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1224,31 +1209,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1260,13 +1227,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1278,7 +1239,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1409,17 +1430,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1435,6 +1450,21 @@
       </top>
       <bottom style="double">
         <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1473,166 +1503,157 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1699,9 +1720,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1726,13 +1744,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2121,7 +2136,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A3:H404"/>
+  <dimension ref="A3:H405"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="14.1428571428571" customWidth="1"/>
@@ -2794,1313 +2809,1346 @@
       </c>
     </row>
     <row r="46" spans="2:6">
-      <c r="B46" s="22"/>
-      <c r="C46" s="23">
+      <c r="B46" s="13"/>
+      <c r="C46" s="22">
         <v>46133</v>
       </c>
-      <c r="D46" s="22" t="s">
+      <c r="D46" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="E46" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F46" s="24" t="s">
+      <c r="E46" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="23" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="47" spans="2:6">
-      <c r="B47" s="22"/>
-      <c r="C47" s="23">
+      <c r="B47" s="13"/>
+      <c r="C47" s="22">
         <v>46140</v>
       </c>
-      <c r="D47" s="22" t="s">
+      <c r="D47" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="E47" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" s="24" t="s">
+      <c r="E47" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="23" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="48" spans="5:5">
-      <c r="E48" s="26"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5">
-      <c r="E49" s="26"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="52" spans="2:6">
-      <c r="B52" s="22" t="s">
+      <c r="B52" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="C52" s="27">
+      <c r="C52" s="26">
         <v>46141</v>
       </c>
-      <c r="D52" s="28" t="s">
+      <c r="D52" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="E52" s="29" t="s">
-        <v>13</v>
-      </c>
-      <c r="F52" s="30" t="s">
+      <c r="E52" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" s="29" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="53" spans="2:6">
-      <c r="B53" s="22"/>
-      <c r="C53" s="31"/>
-      <c r="D53" s="31"/>
-      <c r="E53" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F53" s="30" t="s">
+      <c r="B53" s="13"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="27"/>
+      <c r="E53" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" s="29" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="54" customHeight="1" spans="2:6">
-      <c r="B54" s="22"/>
-      <c r="C54" s="31"/>
-      <c r="D54" s="31"/>
-      <c r="E54" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F54" s="30" t="s">
+      <c r="B54" s="13"/>
+      <c r="C54" s="27"/>
+      <c r="D54" s="27"/>
+      <c r="E54" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" s="29" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="55" spans="2:6">
-      <c r="B55" s="22"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="31"/>
-      <c r="E55" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F55" s="30" t="s">
+      <c r="B55" s="13"/>
+      <c r="C55" s="27"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" s="29" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="56" spans="2:6">
-      <c r="B56" s="22"/>
-      <c r="C56" s="31"/>
-      <c r="D56" s="31"/>
-      <c r="E56" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" s="30" t="s">
+      <c r="B56" s="13"/>
+      <c r="C56" s="27"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" s="29" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="57" spans="2:6">
-      <c r="B57" s="22"/>
-      <c r="C57" s="31"/>
-      <c r="D57" s="31"/>
-      <c r="E57" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F57" s="30" t="s">
+      <c r="B57" s="13"/>
+      <c r="C57" s="27"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F57" s="29" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="58" spans="2:6">
-      <c r="B58" s="22"/>
-      <c r="C58" s="31"/>
-      <c r="D58" s="31"/>
-      <c r="E58" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F58" s="30" t="s">
+      <c r="B58" s="13"/>
+      <c r="C58" s="27"/>
+      <c r="D58" s="27"/>
+      <c r="E58" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" s="29" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="59" spans="2:6">
-      <c r="B59" s="22"/>
-      <c r="C59" s="31"/>
-      <c r="D59" s="28" t="s">
+      <c r="B59" s="13"/>
+      <c r="C59" s="27"/>
+      <c r="D59" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="E59" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F59" s="32" t="s">
+      <c r="E59" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F59" s="30" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="60" spans="2:6">
-      <c r="B60" s="22"/>
-      <c r="C60" s="31"/>
-      <c r="D60" s="33" t="s">
+      <c r="B60" s="13"/>
+      <c r="C60" s="27"/>
+      <c r="D60" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="E60" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F60" s="32" t="s">
+      <c r="E60" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="30" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="61" spans="2:6">
-      <c r="B61" s="22"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="33" t="s">
+      <c r="B61" s="13"/>
+      <c r="C61" s="27"/>
+      <c r="D61" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="E61" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F61" s="32" t="s">
+      <c r="E61" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F61" s="30" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="62" spans="2:6">
-      <c r="B62" s="22"/>
-      <c r="C62" s="31"/>
-      <c r="D62" s="33" t="s">
+      <c r="B62" s="13"/>
+      <c r="C62" s="27"/>
+      <c r="D62" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="E62" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F62" s="32" t="s">
+      <c r="E62" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F62" s="30" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="314" ht="15.75"/>
-    <row r="315" ht="15.75" spans="3:6">
-      <c r="C315" s="34" t="s">
+    <row r="63" spans="3:6">
+      <c r="C63" s="31">
+        <v>46142</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D315" s="35" t="s">
+      <c r="F63" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E315" s="35" t="s">
+    </row>
+    <row r="64" spans="3:6">
+      <c r="C64" s="31"/>
+      <c r="F64" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="F315" s="36" t="s">
+    </row>
+    <row r="65" spans="4:6">
+      <c r="D65" s="2" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="316" spans="3:6">
-      <c r="C316" s="37">
+      <c r="F65" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="66" spans="4:6">
+      <c r="D66" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="315" ht="15.75"/>
+    <row r="316" ht="15.75" spans="3:6">
+      <c r="C316" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="D316" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="E316" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="F316" s="34" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="317" ht="15.75" spans="3:6">
+      <c r="C317" s="35">
         <v>46092</v>
       </c>
-      <c r="D316" s="38" t="s">
+      <c r="D317" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="E316" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F316" s="39" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="317" spans="3:6">
-      <c r="C317" s="40"/>
-      <c r="D317" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="E317" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F317" s="39" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="318" spans="3:6">
-      <c r="C318" s="41"/>
-      <c r="D318" s="38" t="s">
-        <v>122</v>
-      </c>
-      <c r="E318" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F318" s="39" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="319" spans="3:6">
-      <c r="C319" s="37">
+      <c r="E317" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F317" s="37" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="318" ht="15.75" spans="3:6">
+      <c r="C318" s="38"/>
+      <c r="D318" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="E318" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F318" s="37" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="319" ht="15.75" spans="3:6">
+      <c r="C319" s="39"/>
+      <c r="D319" s="36" t="s">
+        <v>129</v>
+      </c>
+      <c r="E319" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F319" s="37" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="320" ht="15.75" spans="3:6">
+      <c r="C320" s="35">
         <v>46093</v>
       </c>
-      <c r="D319" s="38" t="s">
-        <v>124</v>
-      </c>
-      <c r="E319" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F319" s="39" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="320" spans="3:6">
-      <c r="C320" s="40"/>
-      <c r="D320" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="E320" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F320" s="39" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="321" spans="3:6">
-      <c r="C321" s="41"/>
-      <c r="D321" s="38" t="s">
-        <v>128</v>
-      </c>
-      <c r="E321" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F321" s="39" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="322" spans="3:6">
-      <c r="C322" s="42">
+      <c r="D320" s="36" t="s">
+        <v>131</v>
+      </c>
+      <c r="E320" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F320" s="37" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="321" ht="15.75" spans="3:6">
+      <c r="C321" s="38"/>
+      <c r="D321" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="E321" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F321" s="37" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="322" ht="15.75" spans="3:6">
+      <c r="C322" s="39"/>
+      <c r="D322" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="E322" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F322" s="37" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="323" ht="15.75" spans="3:6">
+      <c r="C323" s="40">
         <v>46094</v>
       </c>
-      <c r="D322" s="38" t="s">
+      <c r="D323" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="E322" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F322" s="39" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="323" spans="3:6">
-      <c r="C323" s="43"/>
-      <c r="D323" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="E323" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F323" s="39" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="324" spans="3:6">
-      <c r="C324" s="44"/>
-      <c r="D324" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="E324" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F324" s="39" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="325" spans="3:6">
-      <c r="C325" s="42">
+      <c r="E323" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F323" s="37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="324" ht="15.75" spans="3:6">
+      <c r="C324" s="41"/>
+      <c r="D324" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="E324" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F324" s="37" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="325" ht="15.75" spans="3:6">
+      <c r="C325" s="42"/>
+      <c r="D325" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="E325" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F325" s="37" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="326" ht="15.75" spans="3:6">
+      <c r="C326" s="40">
         <v>46097</v>
       </c>
-      <c r="D325" s="38" t="s">
+      <c r="D326" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="E325" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F325" s="39" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="326" spans="3:6">
-      <c r="C326" s="43"/>
-      <c r="D326" s="38" t="s">
-        <v>136</v>
-      </c>
-      <c r="E326" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F326" s="39" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="327" spans="3:6">
-      <c r="C327" s="44"/>
-      <c r="D327" s="38" t="s">
+      <c r="E326" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F326" s="37" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="327" ht="15.75" spans="3:6">
+      <c r="C327" s="41"/>
+      <c r="D327" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="E327" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F327" s="37" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="328" ht="15.75" spans="3:6">
+      <c r="C328" s="42"/>
+      <c r="D328" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="E327" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F327" s="39" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="328" spans="3:6">
-      <c r="C328" s="42">
+      <c r="E328" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F328" s="37" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="329" ht="15.75" spans="3:6">
+      <c r="C329" s="40">
         <v>46098</v>
       </c>
-      <c r="D328" s="38" t="s">
-        <v>139</v>
-      </c>
-      <c r="E328" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F328" s="39" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="329" spans="3:6">
-      <c r="C329" s="43"/>
-      <c r="D329" s="38" t="s">
-        <v>141</v>
-      </c>
-      <c r="E329" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F329" s="39" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="330" spans="3:6">
-      <c r="C330" s="44"/>
-      <c r="D330" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="E330" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F330" s="39" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="331" spans="3:6">
-      <c r="C331" s="42">
+      <c r="D329" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="E329" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F329" s="37" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="330" ht="15.75" spans="3:6">
+      <c r="C330" s="41"/>
+      <c r="D330" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="E330" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F330" s="37" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="331" ht="15.75" spans="3:6">
+      <c r="C331" s="42"/>
+      <c r="D331" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="E331" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F331" s="37" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="332" ht="15.75" spans="3:6">
+      <c r="C332" s="40">
         <v>46099</v>
       </c>
-      <c r="D331" s="38" t="s">
-        <v>145</v>
-      </c>
-      <c r="E331" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F331" s="39" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="332" spans="3:6">
-      <c r="C332" s="43"/>
-      <c r="D332" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="E332" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F332" s="39" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="333" spans="3:6">
-      <c r="C333" s="44"/>
-      <c r="D333" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E333" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F333" s="39" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="334" spans="3:6">
-      <c r="C334" s="42">
+      <c r="D332" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="E332" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F332" s="37" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="333" ht="15.75" spans="3:6">
+      <c r="C333" s="41"/>
+      <c r="D333" s="36" t="s">
+        <v>154</v>
+      </c>
+      <c r="E333" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F333" s="37" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="334" ht="15.75" spans="3:6">
+      <c r="C334" s="42"/>
+      <c r="D334" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="E334" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F334" s="37" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="335" ht="15.75" spans="3:6">
+      <c r="C335" s="40">
         <v>46100</v>
       </c>
-      <c r="D334" s="38" t="s">
+      <c r="D335" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="E334" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F334" s="39" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="335" spans="3:6">
-      <c r="C335" s="43"/>
-      <c r="D335" s="38" t="s">
-        <v>152</v>
-      </c>
-      <c r="E335" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F335" s="39" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="336" spans="3:6">
-      <c r="C336" s="44"/>
-      <c r="D336" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="E336" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F336" s="39" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="337" spans="3:6">
-      <c r="C337" s="42">
+      <c r="E335" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F335" s="37" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="336" ht="15.75" spans="3:6">
+      <c r="C336" s="41"/>
+      <c r="D336" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="E336" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F336" s="37" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="337" ht="15.75" spans="3:6">
+      <c r="C337" s="42"/>
+      <c r="D337" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="E337" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F337" s="37" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="338" ht="15.75" spans="3:6">
+      <c r="C338" s="40">
         <v>46101</v>
       </c>
-      <c r="D337" s="38" t="s">
+      <c r="D338" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E337" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F337" s="39" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="338" spans="3:6">
-      <c r="C338" s="43"/>
-      <c r="D338" s="38" t="s">
-        <v>157</v>
-      </c>
-      <c r="E338" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F338" s="39" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="339" spans="3:6">
-      <c r="C339" s="44"/>
-      <c r="D339" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="E339" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F339" s="39" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="340" spans="3:6">
-      <c r="C340" s="45">
+      <c r="E338" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F338" s="37" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="339" ht="15.75" spans="3:6">
+      <c r="C339" s="41"/>
+      <c r="D339" s="36" t="s">
+        <v>164</v>
+      </c>
+      <c r="E339" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F339" s="37" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="340" ht="15.75" spans="3:6">
+      <c r="C340" s="42"/>
+      <c r="D340" s="36" t="s">
+        <v>166</v>
+      </c>
+      <c r="E340" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F340" s="37" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="341" ht="15.75" spans="3:6">
+      <c r="C341" s="43">
         <v>46104</v>
       </c>
-      <c r="D340" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="E340" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F340" s="39" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="341" spans="3:6">
-      <c r="C341" s="46"/>
-      <c r="D341" s="38" t="s">
-        <v>163</v>
-      </c>
-      <c r="E341" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F341" s="39" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="342" spans="3:6">
-      <c r="C342" s="47"/>
-      <c r="D342" s="38" t="s">
-        <v>165</v>
-      </c>
-      <c r="E342" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F342" s="39" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="343" spans="3:6">
-      <c r="C343" s="45">
+      <c r="D341" s="36" t="s">
+        <v>168</v>
+      </c>
+      <c r="E341" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F341" s="37" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="342" ht="15.75" spans="3:6">
+      <c r="C342" s="44"/>
+      <c r="D342" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="E342" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F342" s="37" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="343" ht="15.75" spans="3:6">
+      <c r="C343" s="45"/>
+      <c r="D343" s="36" t="s">
+        <v>172</v>
+      </c>
+      <c r="E343" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F343" s="37" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="344" ht="15.75" spans="3:6">
+      <c r="C344" s="43">
         <v>46105</v>
       </c>
-      <c r="D343" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="E343" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F343" s="39" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="344" spans="3:6">
-      <c r="C344" s="46"/>
-      <c r="D344" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="E344" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F344" s="39" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="345" spans="3:6">
-      <c r="C345" s="47"/>
-      <c r="D345" s="38" t="s">
-        <v>171</v>
-      </c>
-      <c r="E345" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F345" s="39" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="346" spans="3:6">
-      <c r="C346" s="45">
+      <c r="D344" s="36" t="s">
+        <v>174</v>
+      </c>
+      <c r="E344" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F344" s="37" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="345" ht="15.75" spans="3:6">
+      <c r="C345" s="44"/>
+      <c r="D345" s="36" t="s">
+        <v>176</v>
+      </c>
+      <c r="E345" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F345" s="37" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="346" ht="15.75" spans="3:6">
+      <c r="C346" s="45"/>
+      <c r="D346" s="36" t="s">
+        <v>178</v>
+      </c>
+      <c r="E346" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F346" s="37" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="347" ht="15.75" spans="3:6">
+      <c r="C347" s="43">
         <v>46106</v>
       </c>
-      <c r="D346" s="38" t="s">
-        <v>173</v>
-      </c>
-      <c r="E346" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F346" s="39" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="347" spans="3:6">
-      <c r="C347" s="46"/>
-      <c r="D347" s="38" t="s">
+      <c r="D347" s="36" t="s">
+        <v>180</v>
+      </c>
+      <c r="E347" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F347" s="37" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="348" ht="15.75" spans="3:6">
+      <c r="C348" s="44"/>
+      <c r="D348" s="36" t="s">
+        <v>182</v>
+      </c>
+      <c r="E348" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F348" s="37" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="349" ht="15.75" spans="3:6">
+      <c r="C349" s="45"/>
+      <c r="D349" s="36" t="s">
+        <v>184</v>
+      </c>
+      <c r="E349" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F349" s="37" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="350" ht="15.75" spans="3:6">
+      <c r="C350" s="43">
+        <v>46107</v>
+      </c>
+      <c r="D350" s="36" t="s">
+        <v>186</v>
+      </c>
+      <c r="E350" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F350" s="37" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="351" ht="15.75" spans="3:6">
+      <c r="C351" s="44"/>
+      <c r="D351" s="36" t="s">
+        <v>188</v>
+      </c>
+      <c r="E351" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F351" s="37" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="352" ht="15.75" spans="3:6">
+      <c r="C352" s="45"/>
+      <c r="D352" s="36" t="s">
+        <v>189</v>
+      </c>
+      <c r="E352" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F352" s="37" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="353" ht="15.75" spans="3:6">
+      <c r="C353" s="43">
+        <v>46108</v>
+      </c>
+      <c r="D353" s="36" t="s">
+        <v>191</v>
+      </c>
+      <c r="E353" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F353" s="37" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="354" ht="15.75" spans="3:6">
+      <c r="C354" s="44"/>
+      <c r="D354" s="36" t="s">
+        <v>193</v>
+      </c>
+      <c r="E354" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F354" s="37" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="355" ht="15.75" spans="3:6">
+      <c r="C355" s="45"/>
+      <c r="D355" s="36" t="s">
+        <v>195</v>
+      </c>
+      <c r="E355" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F355" s="37" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="356" ht="15.75" spans="3:6">
+      <c r="C356" s="43">
+        <v>46111</v>
+      </c>
+      <c r="D356" s="36" t="s">
+        <v>197</v>
+      </c>
+      <c r="E356" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F356" s="46" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="357" ht="15.75" spans="3:6">
+      <c r="C357" s="44"/>
+      <c r="D357" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="E357" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F357" s="46" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="358" ht="15.75" spans="3:6">
+      <c r="C358" s="45"/>
+      <c r="D358" s="36" t="s">
+        <v>201</v>
+      </c>
+      <c r="E358" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F358" s="46" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="359" ht="15.75" spans="3:6">
+      <c r="C359" s="43">
+        <v>46112</v>
+      </c>
+      <c r="D359" s="36" t="s">
+        <v>203</v>
+      </c>
+      <c r="E359" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F359" s="46" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="360" ht="15.75" spans="3:6">
+      <c r="C360" s="44"/>
+      <c r="D360" s="36" t="s">
+        <v>205</v>
+      </c>
+      <c r="E360" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F360" s="46" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="361" ht="15.75" spans="3:6">
+      <c r="C361" s="44"/>
+      <c r="D361" s="36" t="s">
+        <v>207</v>
+      </c>
+      <c r="E361" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F361" s="46" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="362" ht="15.75" spans="3:6">
+      <c r="C362" s="45"/>
+      <c r="D362" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="E362" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F362" s="46" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="363" ht="15.75" spans="3:6">
+      <c r="C363" s="43">
+        <v>46113</v>
+      </c>
+      <c r="D363" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="E363" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F363" s="46" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="364" ht="15.75" spans="3:6">
+      <c r="C364" s="44"/>
+      <c r="D364" s="36" t="s">
+        <v>212</v>
+      </c>
+      <c r="E364" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F364" s="46" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="365" ht="15.75" spans="3:6">
+      <c r="C365" s="45"/>
+      <c r="D365" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="E365" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F365" s="46" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="366" ht="15.75" spans="3:6">
+      <c r="C366" s="43">
+        <v>46114</v>
+      </c>
+      <c r="D366" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="E366" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F366" s="46" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="367" ht="15.75" spans="3:6">
+      <c r="C367" s="44"/>
+      <c r="D367" s="36" t="s">
+        <v>215</v>
+      </c>
+      <c r="E367" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F367" s="46" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="368" ht="15.75" spans="3:6">
+      <c r="C368" s="45"/>
+      <c r="D368" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="E368" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F368" s="46" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="369" ht="15.75" spans="3:6">
+      <c r="C369" s="43">
+        <v>46115</v>
+      </c>
+      <c r="D369" s="36" t="s">
+        <v>218</v>
+      </c>
+      <c r="E369" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F369" s="46" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="370" ht="15.75" spans="3:6">
+      <c r="C370" s="44"/>
+      <c r="D370" s="36" t="s">
+        <v>220</v>
+      </c>
+      <c r="E370" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F370" s="46" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="371" ht="15.75" spans="3:6">
+      <c r="C371" s="45"/>
+      <c r="D371" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="E371" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F371" s="46" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="372" ht="15.75" spans="3:6">
+      <c r="C372" s="40">
+        <v>46118</v>
+      </c>
+      <c r="D372" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="E372" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F372" s="46" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="373" ht="15.75" spans="3:6">
+      <c r="C373" s="41"/>
+      <c r="D373" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="E373" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F373" s="46" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="374" ht="15.75" spans="3:6">
+      <c r="C374" s="41"/>
+      <c r="D374" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="E374" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F374" s="46" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="375" ht="15.75" spans="3:6">
+      <c r="C375" s="42"/>
+      <c r="D375" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="E375" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F375" s="46" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="376" ht="15.75" spans="3:6">
+      <c r="C376" s="40">
+        <v>46119</v>
+      </c>
+      <c r="D376" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="E376" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F376" s="46" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="377" ht="15.75" spans="3:6">
+      <c r="C377" s="41"/>
+      <c r="D377" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="E377" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F377" s="46" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="378" ht="15.75" spans="3:6">
+      <c r="C378" s="42"/>
+      <c r="D378" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="E378" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F378" s="46" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="379" ht="15.75" spans="3:6">
+      <c r="C379" s="40">
+        <v>46120</v>
+      </c>
+      <c r="D379" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="E379" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F379" s="46" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="380" ht="15.75" spans="3:6">
+      <c r="C380" s="41"/>
+      <c r="D380" s="36" t="s">
+        <v>238</v>
+      </c>
+      <c r="E380" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F380" s="46" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="381" ht="15.75" spans="3:6">
+      <c r="C381" s="42"/>
+      <c r="D381" s="36" t="s">
+        <v>240</v>
+      </c>
+      <c r="E381" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F381" s="46" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="382" ht="15.75" spans="3:6">
+      <c r="C382" s="43">
+        <v>46121</v>
+      </c>
+      <c r="D382" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="E382" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F382" s="46" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="383" ht="15.75" spans="3:6">
+      <c r="C383" s="44"/>
+      <c r="D383" s="36" t="s">
+        <v>243</v>
+      </c>
+      <c r="E383" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F383" s="46" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="384" ht="15.75" spans="3:6">
+      <c r="C384" s="45"/>
+      <c r="D384" s="36" t="s">
+        <v>245</v>
+      </c>
+      <c r="E384" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F384" s="46" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="385" ht="15.75" spans="3:6">
+      <c r="C385" s="40">
+        <v>46122</v>
+      </c>
+      <c r="D385" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E385" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F385" s="46" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="386" ht="15.75" spans="3:6">
+      <c r="C386" s="41"/>
+      <c r="D386" s="36" t="s">
+        <v>248</v>
+      </c>
+      <c r="E386" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F386" s="46" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="387" ht="15.75" spans="3:6">
+      <c r="C387" s="42"/>
+      <c r="D387" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="E387" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F387" s="46" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="388" ht="15.75" spans="3:6">
+      <c r="C388" s="43">
+        <v>46125</v>
+      </c>
+      <c r="D388" s="36" t="s">
+        <v>73</v>
+      </c>
+      <c r="E388" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F388" s="46" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="389" ht="15.75" spans="3:6">
+      <c r="C389" s="44"/>
+      <c r="D389" s="36" t="s">
+        <v>253</v>
+      </c>
+      <c r="E389" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F389" s="46" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="390" ht="15.75" spans="3:6">
+      <c r="C390" s="45"/>
+      <c r="D390" s="36" t="s">
+        <v>255</v>
+      </c>
+      <c r="E390" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F390" s="46" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="391" ht="15.75" spans="3:6">
+      <c r="C391" s="43">
+        <v>46126</v>
+      </c>
+      <c r="D391" s="36" t="s">
+        <v>257</v>
+      </c>
+      <c r="E391" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F391" s="46" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="392" ht="15.75" spans="3:6">
+      <c r="C392" s="44"/>
+      <c r="D392" s="36" t="s">
+        <v>259</v>
+      </c>
+      <c r="E392" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F392" s="46" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="393" ht="15.75" spans="3:6">
+      <c r="C393" s="45"/>
+      <c r="D393" s="36" t="s">
+        <v>261</v>
+      </c>
+      <c r="E393" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F393" s="46" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="394" ht="15.75" spans="3:6">
+      <c r="C394" s="40">
+        <v>46127</v>
+      </c>
+      <c r="D394" s="36" t="s">
+        <v>75</v>
+      </c>
+      <c r="E394" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F394" s="46" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="395" ht="15.75" spans="3:6">
+      <c r="C395" s="41"/>
+      <c r="D395" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="E395" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F395" s="46" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="396" ht="15.75" spans="3:6">
+      <c r="C396" s="41"/>
+      <c r="D396" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="E396" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F396" s="46" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="397" ht="15.75" spans="3:6">
+      <c r="C397" s="41"/>
+      <c r="D397" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="E397" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F397" s="46" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="398" ht="15.75" spans="3:6">
+      <c r="C398" s="42"/>
+      <c r="D398" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="E398" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F398" s="46" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="399" ht="15.75" spans="3:6">
+      <c r="C399" s="43">
+        <v>46128</v>
+      </c>
+      <c r="D399" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="E399" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F399" s="46" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="400" ht="15.75" spans="3:6">
+      <c r="C400" s="44"/>
+      <c r="D400" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="E400" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F400" s="46" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="401" ht="15.75" spans="3:6">
+      <c r="C401" s="45"/>
+      <c r="D401" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="E401" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F401" s="46" t="s">
         <v>175</v>
       </c>
-      <c r="E347" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F347" s="39" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="348" spans="3:6">
-      <c r="C348" s="47"/>
-      <c r="D348" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="E348" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F348" s="39" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="349" spans="3:6">
-      <c r="C349" s="45">
-        <v>46107</v>
-      </c>
-      <c r="D349" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="E349" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F349" s="39" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="350" spans="3:6">
-      <c r="C350" s="46"/>
-      <c r="D350" s="38" t="s">
-        <v>181</v>
-      </c>
-      <c r="E350" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F350" s="39" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="351" spans="3:6">
-      <c r="C351" s="47"/>
-      <c r="D351" s="38" t="s">
-        <v>182</v>
-      </c>
-      <c r="E351" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F351" s="39" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="352" spans="3:6">
-      <c r="C352" s="45">
-        <v>46108</v>
-      </c>
-      <c r="D352" s="38" t="s">
-        <v>184</v>
-      </c>
-      <c r="E352" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F352" s="39" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="353" spans="3:6">
-      <c r="C353" s="46"/>
-      <c r="D353" s="38" t="s">
-        <v>186</v>
-      </c>
-      <c r="E353" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F353" s="39" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="354" spans="3:6">
-      <c r="C354" s="47"/>
-      <c r="D354" s="38" t="s">
-        <v>188</v>
-      </c>
-      <c r="E354" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F354" s="39" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="355" spans="3:6">
-      <c r="C355" s="45">
-        <v>46111</v>
-      </c>
-      <c r="D355" s="38" t="s">
-        <v>190</v>
-      </c>
-      <c r="E355" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F355" s="48" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="356" spans="3:6">
-      <c r="C356" s="46"/>
-      <c r="D356" s="38" t="s">
-        <v>192</v>
-      </c>
-      <c r="E356" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F356" s="48" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="357" spans="3:6">
-      <c r="C357" s="47"/>
-      <c r="D357" s="38" t="s">
-        <v>194</v>
-      </c>
-      <c r="E357" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F357" s="48" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="358" spans="3:6">
-      <c r="C358" s="45">
-        <v>46112</v>
-      </c>
-      <c r="D358" s="38" t="s">
-        <v>196</v>
-      </c>
-      <c r="E358" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F358" s="48" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="359" spans="3:6">
-      <c r="C359" s="46"/>
-      <c r="D359" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="E359" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F359" s="48" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="360" spans="3:6">
-      <c r="C360" s="46"/>
-      <c r="D360" s="38" t="s">
-        <v>200</v>
-      </c>
-      <c r="E360" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F360" s="48" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="361" spans="3:6">
-      <c r="C361" s="47"/>
-      <c r="D361" s="38" t="s">
-        <v>202</v>
-      </c>
-      <c r="E361" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F361" s="48" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="362" spans="3:6">
-      <c r="C362" s="45">
-        <v>46113</v>
-      </c>
-      <c r="D362" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="E362" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F362" s="48" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="363" spans="3:6">
-      <c r="C363" s="46"/>
-      <c r="D363" s="38" t="s">
-        <v>205</v>
-      </c>
-      <c r="E363" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F363" s="48" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="364" spans="3:6">
-      <c r="C364" s="47"/>
-      <c r="D364" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="E364" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F364" s="48" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="365" spans="3:6">
-      <c r="C365" s="45">
-        <v>46114</v>
-      </c>
-      <c r="D365" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="E365" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F365" s="48" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="366" spans="3:6">
-      <c r="C366" s="46"/>
-      <c r="D366" s="38" t="s">
-        <v>208</v>
-      </c>
-      <c r="E366" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F366" s="48" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="367" spans="3:6">
-      <c r="C367" s="47"/>
-      <c r="D367" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="E367" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F367" s="48" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="368" spans="3:6">
-      <c r="C368" s="45">
-        <v>46115</v>
-      </c>
-      <c r="D368" s="38" t="s">
-        <v>211</v>
-      </c>
-      <c r="E368" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F368" s="48" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="369" spans="3:6">
-      <c r="C369" s="46"/>
-      <c r="D369" s="38" t="s">
-        <v>213</v>
-      </c>
-      <c r="E369" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F369" s="48" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="370" spans="3:6">
-      <c r="C370" s="47"/>
-      <c r="D370" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="E370" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F370" s="48" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="371" spans="3:6">
-      <c r="C371" s="42">
-        <v>46118</v>
-      </c>
-      <c r="D371" s="38" t="s">
-        <v>217</v>
-      </c>
-      <c r="E371" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F371" s="48" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="372" spans="3:6">
-      <c r="C372" s="43"/>
-      <c r="D372" s="38" t="s">
-        <v>219</v>
-      </c>
-      <c r="E372" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F372" s="48" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="373" spans="3:6">
-      <c r="C373" s="43"/>
-      <c r="D373" s="38" t="s">
-        <v>221</v>
-      </c>
-      <c r="E373" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F373" s="48" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="374" spans="3:6">
-      <c r="C374" s="44"/>
-      <c r="D374" s="38" t="s">
-        <v>223</v>
-      </c>
-      <c r="E374" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F374" s="48" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="375" spans="3:6">
-      <c r="C375" s="42">
-        <v>46119</v>
-      </c>
-      <c r="D375" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="E375" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F375" s="48" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="376" spans="3:6">
-      <c r="C376" s="43"/>
-      <c r="D376" s="38" t="s">
-        <v>226</v>
-      </c>
-      <c r="E376" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F376" s="48" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="377" spans="3:6">
-      <c r="C377" s="44"/>
-      <c r="D377" s="38" t="s">
-        <v>228</v>
-      </c>
-      <c r="E377" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F377" s="48" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="378" spans="3:6">
-      <c r="C378" s="42">
-        <v>46120</v>
-      </c>
-      <c r="D378" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="E378" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F378" s="48" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="379" spans="3:6">
-      <c r="C379" s="43"/>
-      <c r="D379" s="38" t="s">
-        <v>231</v>
-      </c>
-      <c r="E379" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F379" s="48" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="380" spans="3:6">
-      <c r="C380" s="44"/>
-      <c r="D380" s="38" t="s">
-        <v>233</v>
-      </c>
-      <c r="E380" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F380" s="48" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="381" spans="3:6">
-      <c r="C381" s="45">
-        <v>46121</v>
-      </c>
-      <c r="D381" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="E381" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F381" s="48" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="382" spans="3:6">
-      <c r="C382" s="46"/>
-      <c r="D382" s="38" t="s">
-        <v>236</v>
-      </c>
-      <c r="E382" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F382" s="48" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="383" spans="3:6">
-      <c r="C383" s="47"/>
-      <c r="D383" s="38" t="s">
-        <v>238</v>
-      </c>
-      <c r="E383" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F383" s="48" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="384" spans="3:6">
-      <c r="C384" s="42">
-        <v>46122</v>
-      </c>
-      <c r="D384" s="38" t="s">
-        <v>69</v>
-      </c>
-      <c r="E384" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F384" s="48" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="385" spans="3:6">
-      <c r="C385" s="43"/>
-      <c r="D385" s="38" t="s">
-        <v>241</v>
-      </c>
-      <c r="E385" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F385" s="48" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="386" spans="3:6">
-      <c r="C386" s="44"/>
-      <c r="D386" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="E386" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F386" s="48" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="387" spans="3:6">
-      <c r="C387" s="45">
-        <v>46125</v>
-      </c>
-      <c r="D387" s="38" t="s">
-        <v>73</v>
-      </c>
-      <c r="E387" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F387" s="48" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="388" spans="3:6">
-      <c r="C388" s="46"/>
-      <c r="D388" s="38" t="s">
-        <v>246</v>
-      </c>
-      <c r="E388" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F388" s="48" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="389" spans="3:6">
-      <c r="C389" s="47"/>
-      <c r="D389" s="38" t="s">
-        <v>248</v>
-      </c>
-      <c r="E389" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F389" s="48" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="390" spans="3:6">
-      <c r="C390" s="45">
-        <v>46126</v>
-      </c>
-      <c r="D390" s="38" t="s">
-        <v>250</v>
-      </c>
-      <c r="E390" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F390" s="48" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="391" spans="3:6">
-      <c r="C391" s="46"/>
-      <c r="D391" s="38" t="s">
-        <v>252</v>
-      </c>
-      <c r="E391" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F391" s="48" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="392" spans="3:6">
-      <c r="C392" s="47"/>
-      <c r="D392" s="38" t="s">
-        <v>254</v>
-      </c>
-      <c r="E392" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F392" s="48" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="393" spans="3:6">
-      <c r="C393" s="42">
-        <v>46127</v>
-      </c>
-      <c r="D393" s="38" t="s">
-        <v>75</v>
-      </c>
-      <c r="E393" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F393" s="48" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="394" spans="3:6">
-      <c r="C394" s="43"/>
-      <c r="D394" s="38" t="s">
-        <v>76</v>
-      </c>
-      <c r="E394" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F394" s="48" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="395" spans="3:6">
-      <c r="C395" s="43"/>
-      <c r="D395" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="E395" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F395" s="48" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="396" spans="3:6">
-      <c r="C396" s="43"/>
-      <c r="D396" s="38" t="s">
-        <v>80</v>
-      </c>
-      <c r="E396" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F396" s="48" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="397" spans="3:6">
-      <c r="C397" s="44"/>
-      <c r="D397" s="38" t="s">
-        <v>82</v>
-      </c>
-      <c r="E397" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F397" s="48" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="398" spans="3:6">
-      <c r="C398" s="45">
-        <v>46128</v>
-      </c>
-      <c r="D398" s="38" t="s">
-        <v>84</v>
-      </c>
-      <c r="E398" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F398" s="48" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="399" spans="3:6">
-      <c r="C399" s="46"/>
-      <c r="D399" s="38" t="s">
-        <v>86</v>
-      </c>
-      <c r="E399" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F399" s="48" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="400" spans="3:6">
-      <c r="C400" s="47"/>
-      <c r="D400" s="38" t="s">
-        <v>88</v>
-      </c>
-      <c r="E400" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F400" s="48" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="401" spans="3:6">
-      <c r="C401" s="45">
+    </row>
+    <row r="402" ht="15.75" spans="3:6">
+      <c r="C402" s="43">
         <v>46129</v>
       </c>
-      <c r="D401" s="38" t="s">
+      <c r="D402" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="E401" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F401" s="48" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="402" spans="3:6">
-      <c r="C402" s="46"/>
-      <c r="D402" s="38" t="s">
-        <v>264</v>
-      </c>
-      <c r="E402" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F402" s="48" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="403" spans="3:6">
-      <c r="C403" s="46"/>
-      <c r="D403" s="38" t="s">
+      <c r="E402" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F402" s="46" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="403" ht="15.75" spans="3:6">
+      <c r="C403" s="44"/>
+      <c r="D403" s="36" t="s">
+        <v>271</v>
+      </c>
+      <c r="E403" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F403" s="46" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="404" ht="15.75" spans="3:6">
+      <c r="C404" s="44"/>
+      <c r="D404" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="E403" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F403" s="48" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="404" spans="3:6">
-      <c r="C404" s="47"/>
-      <c r="D404" s="38" t="s">
-        <v>267</v>
-      </c>
-      <c r="E404" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F404" s="48" t="s">
-        <v>268</v>
+      <c r="E404" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F404" s="46" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="405" ht="15.75" spans="3:6">
+      <c r="C405" s="45"/>
+      <c r="D405" s="36" t="s">
+        <v>274</v>
+      </c>
+      <c r="E405" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F405" s="46" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -4108,41 +4156,41 @@
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B9:B27"/>
     <mergeCell ref="B29:B45"/>
-    <mergeCell ref="C316:C318"/>
-    <mergeCell ref="C319:C321"/>
-    <mergeCell ref="C322:C324"/>
-    <mergeCell ref="C325:C327"/>
-    <mergeCell ref="C328:C330"/>
-    <mergeCell ref="C331:C333"/>
-    <mergeCell ref="C334:C336"/>
-    <mergeCell ref="C337:C339"/>
-    <mergeCell ref="C340:C342"/>
-    <mergeCell ref="C343:C345"/>
-    <mergeCell ref="C346:C348"/>
-    <mergeCell ref="C349:C351"/>
-    <mergeCell ref="C352:C354"/>
-    <mergeCell ref="C355:C357"/>
-    <mergeCell ref="C358:C361"/>
-    <mergeCell ref="C362:C364"/>
-    <mergeCell ref="C365:C367"/>
-    <mergeCell ref="C368:C370"/>
-    <mergeCell ref="C371:C374"/>
-    <mergeCell ref="C375:C377"/>
-    <mergeCell ref="C378:C380"/>
-    <mergeCell ref="C381:C383"/>
-    <mergeCell ref="C384:C386"/>
-    <mergeCell ref="C387:C389"/>
-    <mergeCell ref="C390:C392"/>
-    <mergeCell ref="C393:C397"/>
-    <mergeCell ref="C398:C400"/>
-    <mergeCell ref="C401:C404"/>
+    <mergeCell ref="C317:C319"/>
+    <mergeCell ref="C320:C322"/>
+    <mergeCell ref="C323:C325"/>
+    <mergeCell ref="C326:C328"/>
+    <mergeCell ref="C329:C331"/>
+    <mergeCell ref="C332:C334"/>
+    <mergeCell ref="C335:C337"/>
+    <mergeCell ref="C338:C340"/>
+    <mergeCell ref="C341:C343"/>
+    <mergeCell ref="C344:C346"/>
+    <mergeCell ref="C347:C349"/>
+    <mergeCell ref="C350:C352"/>
+    <mergeCell ref="C353:C355"/>
+    <mergeCell ref="C356:C358"/>
+    <mergeCell ref="C359:C362"/>
+    <mergeCell ref="C363:C365"/>
+    <mergeCell ref="C366:C368"/>
+    <mergeCell ref="C369:C371"/>
+    <mergeCell ref="C372:C375"/>
+    <mergeCell ref="C376:C378"/>
+    <mergeCell ref="C379:C381"/>
+    <mergeCell ref="C382:C384"/>
+    <mergeCell ref="C385:C387"/>
+    <mergeCell ref="C388:C390"/>
+    <mergeCell ref="C391:C393"/>
+    <mergeCell ref="C394:C398"/>
+    <mergeCell ref="C399:C401"/>
+    <mergeCell ref="C402:C405"/>
   </mergeCells>
   <conditionalFormatting sqref="E4:E29">
     <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
       <formula>"Completed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:E45 E64:E65 E156:E314 E405:E1048576">
+  <conditionalFormatting sqref="E1:E45 E65:E66 E406:E1048576 E157:E315">
     <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"Completed"</formula>
     </cfRule>

</xml_diff>